<commit_message>
Add local Amount row to see multiple currency
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,15 +511,25 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>original_amount</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>original_currency</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>payer</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>is_reimbursement</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
@@ -548,15 +558,23 @@
           <t>EUR</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="H2" t="b">
+      <c r="J2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>FOOD</t>
         </is>
@@ -573,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -617,6 +635,16 @@
           <t>currency</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>original_share</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>original_currency</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -650,6 +678,14 @@
         <v>15</v>
       </c>
       <c r="I2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>

<commit_message>
Export all parsed fields and warn on paginated responses
- Add type_transaction column to entries and allocations sheets so
  INCOME, NORMAL, and BALANCE entries are distinguishable (fixes #38)
- Add created, status, type columns to entries sheet and split_type,
  share_ratio columns to allocations sheet (fixes #39)
- Detect paginated API responses and print a warning when the export
  may be incomplete (fixes #40)
- Regenerate reference Excel fixtures to match new output format
- Add 9 targeted tests covering the new columns and pagination warning

Generated with Devin (https://cli.devin.ai/docs)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
+++ b/tricount_extractor/tests/data/expected_results/attachment_test_4.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,45 +491,65 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>created</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>amount</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>original_amount</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>original_currency</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>payer</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>is_reimbursement</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>type_transaction</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
@@ -545,36 +565,54 @@
       <c r="C2" s="1" t="n">
         <v>45658.5</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="n">
+        <v>45658.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Receipt</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="J2" t="b">
+      <c r="K2" t="b">
         <v>0</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>FOOD</t>
         </is>
@@ -591,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,27 +660,42 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>type_transaction</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>participant</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>share</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>original_share</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>original_currency</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>split_type</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>share_ratio</t>
         </is>
       </c>
     </row>
@@ -671,24 +724,37 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>15</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>RATIO</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>